<commit_message>
Boolean Queries and Date Ranges
The exact Boolean search queries used for each database (e.g., Scopus, Web of Science, IEEE Xplore), along with the date ranges covered for each search, ensuring reproducibility of the literature search.
</commit_message>
<xml_diff>
--- a/Boolean_query_date_rage.xlsx
+++ b/Boolean_query_date_rage.xlsx
@@ -1,35 +1,149 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375"/>
+    <workbookView windowHeight="17655"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+  <si>
+    <t>Database</t>
+  </si>
+  <si>
+    <t>Links</t>
+  </si>
+  <si>
+    <t>Search Period</t>
+  </si>
+  <si>
+    <t>Last Accessed</t>
+  </si>
+  <si>
+    <t>Results Found</t>
+  </si>
+  <si>
+    <t>ACM Digital Library</t>
+  </si>
+  <si>
+    <t>https://dl.acm.org/</t>
+  </si>
+  <si>
+    <t>Jan 2018 – Jul 2025</t>
+  </si>
+  <si>
+    <t>IEEE Xplore</t>
+  </si>
+  <si>
+    <t>https://ieeexplore.ieee.org/Xplore/home.jsp</t>
+  </si>
+  <si>
+    <t>Web of Science</t>
+  </si>
+  <si>
+    <t>https://webofscience.clarivate.cn/wos/woscc/basic-search</t>
+  </si>
+  <si>
+    <t>Scopus</t>
+  </si>
+  <si>
+    <t>https://www.scopus.com/pages/home#basic</t>
+  </si>
+  <si>
+    <t>ScienceDirect</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/search</t>
+  </si>
+  <si>
+    <t>Springer</t>
+  </si>
+  <si>
+    <t>https://www.springer.com/gp</t>
+  </si>
+  <si>
+    <t>Boolean Query:</t>
+  </si>
+  <si>
+    <t>("adversarial attack" OR "adversarial example" OR "adversarial patch") AND ("physical" OR "real world") AND ("camouflage" OR "optical" OR "light" OR "illumination" OR "laser" OR "infrared" OR "camera" OR "sensor")</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF0F1115"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000033"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10.5"/>
+      <color rgb="FF000033"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -176,7 +290,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -185,6 +299,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -370,12 +496,64 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="13">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -496,139 +674,175 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -689,6 +903,13 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
+<customStorage xmlns="https://web.wps.cn/et/2018/main">
+  <book/>
+  <sheets/>
+</customStorage>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -941,33 +1162,166 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
-  <sheetData/>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="27.125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="64" style="2" customWidth="1"/>
+    <col min="3" max="3" width="34.5" style="2" customWidth="1"/>
+    <col min="4" max="4" width="29.625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="49.625" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:5">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" customHeight="1" spans="1:5">
+      <c r="A2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="6">
+        <v>45841</v>
+      </c>
+      <c r="E2" s="7">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" customHeight="1" spans="1:5">
+      <c r="A3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6">
+        <v>45841</v>
+      </c>
+      <c r="E3" s="7">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="4" customHeight="1" spans="1:5">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6">
+        <v>45843</v>
+      </c>
+      <c r="E4" s="7">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" customHeight="1" spans="1:5">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="6">
+        <v>45844</v>
+      </c>
+      <c r="E5" s="7">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="6" customHeight="1" spans="1:7">
+      <c r="A6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="6">
+        <v>45848</v>
+      </c>
+      <c r="E6" s="7">
+        <v>152</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" customHeight="1" spans="1:5">
+      <c r="A7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="6">
+        <v>45848</v>
+      </c>
+      <c r="E7" s="7">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" spans="1:5">
+      <c r="A8" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="11"/>
+    </row>
+    <row r="9" customHeight="1" spans="3:3">
+      <c r="C9" s="12"/>
+    </row>
+    <row r="10" customHeight="1" spans="3:3">
+      <c r="C10" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B8:E8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://dl.acm.org/" tooltip="https://dl.acm.org/}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://ieeexplore.ieee.org/Xplore/home.jsp" tooltip="https://ieeexplore.ieee.org/Xplore/home.jsp}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://webofscience.clarivate.cn/wos/woscc/basic-search" tooltip="https://webofscience.clarivate.cn/wos/woscc/basic-search}"/>
+    <hyperlink ref="B5" r:id="rId4" location="basic}" display="https://www.scopus.com/pages/home#basic"/>
+    <hyperlink ref="B6" r:id="rId5" display="https://www.sciencedirect.com/search" tooltip="https://www.sciencedirect.com/search}"/>
+    <hyperlink ref="B7" r:id="rId6" display="https://www.springer.com/gp" tooltip="https://www.springer.com/gp}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>